<commit_message>
Add YAML-driven candidate selection with CLI, highlight candidates on map, drop DB dependency from get_data.py
</commit_message>
<xml_diff>
--- a/data/processed/candidates_summary/candidates_summary.xlsx
+++ b/data/processed/candidates_summary/candidates_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,14 +533,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LORA</t>
+          <t>EIND</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -557,13 +557,13 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>1419</v>
+        <v>1404</v>
       </c>
       <c r="F4" t="n">
-        <v>1386</v>
+        <v>1381</v>
       </c>
       <c r="G4" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -614,7 +614,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RBEY</t>
+          <t>LORA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -624,34 +624,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>1263</v>
+        <v>1419</v>
       </c>
       <c r="F6" t="n">
-        <v>1015</v>
+        <v>1386</v>
       </c>
       <c r="G6" t="n">
-        <v>248</v>
+        <v>33</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RBEY</t>
+          <t>LORA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -661,34 +661,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>1263</v>
+        <v>1419</v>
       </c>
       <c r="F7" t="n">
-        <v>1015</v>
+        <v>1386</v>
       </c>
       <c r="G7" t="n">
-        <v>248</v>
+        <v>33</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RAKT</t>
+          <t>RBEY</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -698,20 +698,20 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D8" t="n">
         <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>1317</v>
+        <v>1263</v>
       </c>
       <c r="F8" t="n">
-        <v>1303</v>
+        <v>1015</v>
       </c>
       <c r="G8" t="n">
-        <v>14</v>
+        <v>248</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -725,7 +725,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RAKT</t>
+          <t>RBEY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -735,76 +735,76 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>1317</v>
+        <v>1263</v>
       </c>
       <c r="F9" t="n">
-        <v>1303</v>
+        <v>1015</v>
       </c>
       <c r="G9" t="n">
-        <v>14</v>
+        <v>248</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PZHT</t>
+          <t>RBEY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07-12-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>1135</v>
+        <v>1263</v>
       </c>
       <c r="F10" t="n">
-        <v>1130</v>
+        <v>1015</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
+        <v>248</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PZHT</t>
+          <t>RAKT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07-12-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -813,35 +813,35 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>1135</v>
+        <v>1317</v>
       </c>
       <c r="F11" t="n">
-        <v>1130</v>
+        <v>1303</v>
       </c>
       <c r="G11" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DYRG</t>
+          <t>RAKT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>27-06-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -853,13 +853,13 @@
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>1423</v>
+        <v>1317</v>
       </c>
       <c r="F12" t="n">
-        <v>1402</v>
+        <v>1303</v>
       </c>
       <c r="G12" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -873,12 +873,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DYRG</t>
+          <t>RAKT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>27-06-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -890,32 +890,32 @@
         <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>1423</v>
+        <v>1317</v>
       </c>
       <c r="F13" t="n">
-        <v>1402</v>
+        <v>1303</v>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NARS</t>
+          <t>PZHT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12-07-2022</t>
+          <t>07-12-2022</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -924,35 +924,35 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="E14" t="n">
-        <v>1165</v>
+        <v>1135</v>
       </c>
       <c r="F14" t="n">
-        <v>1154</v>
+        <v>1130</v>
       </c>
       <c r="G14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NARS</t>
+          <t>PZHT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>12-07-2022</t>
+          <t>07-12-2022</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -961,16 +961,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="E15" t="n">
-        <v>1165</v>
+        <v>1135</v>
       </c>
       <c r="F15" t="n">
-        <v>1154</v>
+        <v>1130</v>
       </c>
       <c r="G15" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -984,12 +984,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DBOZ</t>
+          <t>PZHT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>07-12-2022</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -998,35 +998,35 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="E16" t="n">
-        <v>1423</v>
+        <v>1135</v>
       </c>
       <c r="F16" t="n">
-        <v>1411</v>
+        <v>1130</v>
       </c>
       <c r="G16" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DBOZ</t>
+          <t>DYRG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>27-06-2022</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1041,10 +1041,10 @@
         <v>1423</v>
       </c>
       <c r="F17" t="n">
-        <v>1411</v>
+        <v>1402</v>
       </c>
       <c r="G17" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1058,30 +1058,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CKSH</t>
+          <t>DYRG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>27-06-2022</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>1278</v>
+        <v>1423</v>
       </c>
       <c r="F18" t="n">
-        <v>1266</v>
+        <v>1402</v>
       </c>
       <c r="G18" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1095,49 +1095,49 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CKSH</t>
+          <t>DYRG</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>27-06-2022</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>1278</v>
+        <v>1423</v>
       </c>
       <c r="F19" t="n">
-        <v>1266</v>
+        <v>1402</v>
       </c>
       <c r="G19" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PUZK</t>
+          <t>NARS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>12-07-2022</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1149,13 +1149,13 @@
         <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>1359</v>
+        <v>1165</v>
       </c>
       <c r="F20" t="n">
-        <v>1342</v>
+        <v>1154</v>
       </c>
       <c r="G20" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1169,12 +1169,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PUZK</t>
+          <t>NARS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>12-07-2022</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1186,13 +1186,13 @@
         <v>4</v>
       </c>
       <c r="E21" t="n">
-        <v>1359</v>
+        <v>1165</v>
       </c>
       <c r="F21" t="n">
-        <v>1342</v>
+        <v>1154</v>
       </c>
       <c r="G21" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1206,12 +1206,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TNIS</t>
+          <t>NARS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28-06-2022</t>
+          <t>12-07-2022</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1223,13 +1223,13 @@
         <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>1380</v>
+        <v>1165</v>
       </c>
       <c r="F22" t="n">
-        <v>1371</v>
+        <v>1154</v>
       </c>
       <c r="G22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1243,7 +1243,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TNIS</t>
+          <t>DBOZ</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1260,27 +1260,27 @@
         <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>1380</v>
+        <v>1423</v>
       </c>
       <c r="F23" t="n">
-        <v>1371</v>
+        <v>1411</v>
       </c>
       <c r="G23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MKRJ</t>
+          <t>DBOZ</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1297,10 +1297,10 @@
         <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>1434</v>
+        <v>1423</v>
       </c>
       <c r="F24" t="n">
-        <v>1422</v>
+        <v>1411</v>
       </c>
       <c r="G24" t="n">
         <v>12</v>
@@ -1317,7 +1317,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MKRJ</t>
+          <t>DBOZ</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1334,10 +1334,10 @@
         <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>1434</v>
+        <v>1423</v>
       </c>
       <c r="F25" t="n">
-        <v>1422</v>
+        <v>1411</v>
       </c>
       <c r="G25" t="n">
         <v>12</v>
@@ -1347,14 +1347,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MSAT</t>
+          <t>CKSH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1364,20 +1364,20 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D26" t="n">
         <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>1408</v>
+        <v>1278</v>
       </c>
       <c r="F26" t="n">
-        <v>1384</v>
+        <v>1266</v>
       </c>
       <c r="G26" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1391,7 +1391,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MSAT</t>
+          <t>CKSH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1401,39 +1401,39 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>1408</v>
+        <v>1278</v>
       </c>
       <c r="F27" t="n">
-        <v>1384</v>
+        <v>1266</v>
       </c>
       <c r="G27" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MAKD</t>
+          <t>CKSH</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01-09-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1442,146 +1442,146 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
-        <v>1169</v>
+        <v>1278</v>
       </c>
       <c r="F28" t="n">
-        <v>1156</v>
+        <v>1266</v>
       </c>
       <c r="G28" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MAKD</t>
+          <t>PUZK</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01-09-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>1169</v>
+        <v>1359</v>
       </c>
       <c r="F29" t="n">
-        <v>1156</v>
+        <v>1342</v>
       </c>
       <c r="G29" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SEKB</t>
+          <t>PUZK</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>27-06-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D30" t="n">
         <v>4</v>
       </c>
       <c r="E30" t="n">
-        <v>1300</v>
+        <v>1359</v>
       </c>
       <c r="F30" t="n">
-        <v>1288</v>
+        <v>1342</v>
       </c>
       <c r="G30" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SEKB</t>
+          <t>PUZK</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>27-06-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>4</v>
       </c>
       <c r="E31" t="n">
-        <v>1300</v>
+        <v>1359</v>
       </c>
       <c r="F31" t="n">
-        <v>1288</v>
+        <v>1342</v>
       </c>
       <c r="G31" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SSHB</t>
+          <t>TNIS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>17-11-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1590,35 +1590,35 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>1174</v>
+        <v>1380</v>
       </c>
       <c r="F32" t="n">
-        <v>1168</v>
+        <v>1371</v>
       </c>
       <c r="G32" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SSHB</t>
+          <t>TNIS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>17-11-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1627,16 +1627,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="E33" t="n">
-        <v>1174</v>
+        <v>1380</v>
       </c>
       <c r="F33" t="n">
-        <v>1168</v>
+        <v>1371</v>
       </c>
       <c r="G33" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1650,67 +1650,67 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>FCKP</t>
+          <t>TNIS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>18-10-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="E34" t="n">
-        <v>1125</v>
+        <v>1380</v>
       </c>
       <c r="F34" t="n">
-        <v>1114</v>
+        <v>1371</v>
       </c>
       <c r="G34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>FCKP</t>
+          <t>MKRJ</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>18-10-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
-        <v>1125</v>
+        <v>1434</v>
       </c>
       <c r="F35" t="n">
-        <v>1114</v>
+        <v>1422</v>
       </c>
       <c r="G35" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1724,12 +1724,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>BUSH</t>
+          <t>MKRJ</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27-06-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1741,10 +1741,10 @@
         <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>1305</v>
+        <v>1434</v>
       </c>
       <c r="F36" t="n">
-        <v>1293</v>
+        <v>1422</v>
       </c>
       <c r="G36" t="n">
         <v>12</v>
@@ -1754,19 +1754,19 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BUSH</t>
+          <t>MKRJ</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27-06-2022</t>
+          <t>28-06-2022</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1778,10 +1778,10 @@
         <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>1305</v>
+        <v>1434</v>
       </c>
       <c r="F37" t="n">
-        <v>1293</v>
+        <v>1422</v>
       </c>
       <c r="G37" t="n">
         <v>12</v>
@@ -1791,14 +1791,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ZNUR</t>
+          <t>MSAT</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1815,13 +1815,13 @@
         <v>4</v>
       </c>
       <c r="E38" t="n">
-        <v>1375</v>
+        <v>1408</v>
       </c>
       <c r="F38" t="n">
-        <v>1364</v>
+        <v>1384</v>
       </c>
       <c r="G38" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -1835,35 +1835,738 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>MSAT</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>28-06-2022</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1408</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1384</v>
+      </c>
+      <c r="G39" t="n">
+        <v>24</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MSAT</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>28-06-2022</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1408</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1384</v>
+      </c>
+      <c r="G40" t="n">
+        <v>24</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MAKD</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>01-09-2022</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1169</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1156</v>
+      </c>
+      <c r="G41" t="n">
+        <v>10</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MAKD</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>01-09-2022</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1169</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1156</v>
+      </c>
+      <c r="G42" t="n">
+        <v>10</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MAKD</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>01-09-2022</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1169</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1156</v>
+      </c>
+      <c r="G43" t="n">
+        <v>10</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SEKB</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>27-06-2022</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1288</v>
+      </c>
+      <c r="G44" t="n">
+        <v>12</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SEKB</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>27-06-2022</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>4</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1288</v>
+      </c>
+      <c r="G45" t="n">
+        <v>12</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SEKB</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>27-06-2022</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1288</v>
+      </c>
+      <c r="G46" t="n">
+        <v>12</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SSHB</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17-11-2022</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1174</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1168</v>
+      </c>
+      <c r="G47" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SSHB</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>17-11-2022</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1174</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1168</v>
+      </c>
+      <c r="G48" t="n">
+        <v>5</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SSHB</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>17-11-2022</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1174</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1168</v>
+      </c>
+      <c r="G49" t="n">
+        <v>5</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FCKP</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>18-10-2022</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1114</v>
+      </c>
+      <c r="G50" t="n">
+        <v>10</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>FCKP</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>18-10-2022</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1114</v>
+      </c>
+      <c r="G51" t="n">
+        <v>10</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>FCKP</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>18-10-2022</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1114</v>
+      </c>
+      <c r="G52" t="n">
+        <v>10</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BUSH</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>27-06-2022</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>4</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1305</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1293</v>
+      </c>
+      <c r="G53" t="n">
+        <v>12</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page004_idx01.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BUSH</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>27-06-2022</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1305</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1293</v>
+      </c>
+      <c r="G54" t="n">
+        <v>12</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BUSH</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>27-06-2022</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1305</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1293</v>
+      </c>
+      <c r="G55" t="n">
+        <v>12</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>ZNUR</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>28-06-2022</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>11-07-2026</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>4</v>
-      </c>
-      <c r="E39" t="n">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>28-06-2022</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" t="n">
         <v>1375</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F56" t="n">
         <v>1364</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G56" t="n">
         <v>11</v>
       </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="inlineStr">
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>data/processed/QGEO-KZ_Preliminary_Stability_Assessment_MIRASpaco/table_page005_idx01.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ZNUR</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>28-06-2022</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>4</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1375</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1364</v>
+      </c>
+      <c r="G57" t="n">
+        <v>11</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>data/processed/candidates_summary/candidates_summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ZNUR</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>28-06-2022</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1375</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1364</v>
+      </c>
+      <c r="G58" t="n">
+        <v>11</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
         <is>
           <t>data/processed/candidates_summary/candidates_summary.csv</t>
         </is>

</xml_diff>